<commit_message>
added rq3 experiments + correlation analysis script
</commit_message>
<xml_diff>
--- a/data/output/evaluation/apps.xlsx
+++ b/data/output/evaluation/apps.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GESSI\Projectes\llm-recommender-system\data\output\evaluation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83B322D9-B116-4B13-BD83-D5CD6806DA93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE7D4FB8-04BD-4855-B2A0-526661C5E3BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1375" uniqueCount="1372">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1374" uniqueCount="1371">
   <si>
     <t>name</t>
   </si>
@@ -3964,9 +3964,6 @@
   </si>
   <si>
     <t>WhatsApp Business</t>
-  </si>
-  <si>
-    <t>WhatsApp Business API (via providers like Route Mobile, AiSensy, SendPulse)</t>
   </si>
   <si>
     <t>Whiteout Survival</t>
@@ -4458,10 +4455,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C1373"/>
+  <dimension ref="A1:C1372"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="38.28515625" customWidth="1"/>
+    <col min="1" max="1" width="63.140625" customWidth="1"/>
     <col min="2" max="2" width="23.42578125" customWidth="1"/>
     <col min="3" max="3" width="17.42578125" customWidth="1"/>
   </cols>
@@ -11332,11 +11329,6 @@
         <v>1370</v>
       </c>
     </row>
-    <row r="1373" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1373" t="s">
-        <v>1371</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>